<commit_message>
checks for padded cell values
</commit_message>
<xml_diff>
--- a/tests/data/shift_ignore/workbook.xlsx
+++ b/tests/data/shift_ignore/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/shift_ignore/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0649420-EEF9-AE4F-B628-CB50A34B9AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0F32A9-BDB4-2945-95FA-07B8C67A2360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4160" yWindow="24720" windowWidth="28800" windowHeight="15600" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
+    <workbookView xWindow="4440" yWindow="3480" windowWidth="28800" windowHeight="15600" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="page-desc" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>foo</t>
   </si>
@@ -124,6 +124,21 @@
   </si>
   <si>
     <t>grim</t>
+  </si>
+  <si>
+    <t>nuh65</t>
+  </si>
+  <si>
+    <t>jkl</t>
+  </si>
+  <si>
+    <t>glip</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> mssing       </t>
+  </si>
+  <si>
+    <t>this one has spaces</t>
   </si>
 </sst>
 </file>
@@ -496,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58ABCA7-652D-9640-A447-D695C3291F2E}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -568,6 +583,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -576,7 +602,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640D4E5C-A101-794A-8A66-BA19A027AC5F}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="50.6640625" customWidth="1"/>
@@ -657,6 +683,17 @@
         <v>19</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>